<commit_message>
chore: publish full latest working code to main (via GitHub API)
Consolidates the local main history (26 commits, tip ceba9606ff5a) into a single commit whose tree is identical to local HEAD. Published through the REST API because native git push and SSH are blocked by the corporate network.

Includes: margin CSR gate moved to the Kohler-type shower product, order-confirmation card enrichment, audit-trail redesign, radio-button CSR selections, and docs/CSR-Approval-Processes.md.
</commit_message>
<xml_diff>
--- a/mock-data/customer-master-data.xlsx
+++ b/mock-data/customer-master-data.xlsx
@@ -8,10 +8,12 @@
   </bookViews>
   <sheets>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Customer_Master" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Account_Hierarchy" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Ship_To_Master" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Hierarchy_Rules" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Fulfillment_Rules" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Order_History" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Order_History_Lines" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Account_Hierarchy" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Ship_To_Master" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Hierarchy_Rules" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Fulfillment_Rules" sheetId="7" state="visible" r:id="rId7"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -476,7 +478,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J8"/>
+  <dimension ref="A1:M8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -489,6 +491,9 @@
     <col width="14" customWidth="1" min="8" max="8"/>
     <col width="12" customWidth="1" min="9" max="9"/>
     <col width="14" customWidth="1" min="10" max="10"/>
+    <col width="16" customWidth="1" min="11" max="11"/>
+    <col width="22" customWidth="1" min="12" max="12"/>
+    <col width="14" customWidth="1" min="13" max="13"/>
   </cols>
   <sheetData>
     <row r="1" ht="26" customHeight="1">
@@ -546,6 +551,21 @@
       </c>
       <c r="J2" s="2" t="inlineStr">
         <is>
+          <t>payment_terms</t>
+        </is>
+      </c>
+      <c r="K2" s="2" t="inlineStr">
+        <is>
+          <t>customer_class</t>
+        </is>
+      </c>
+      <c r="L2" s="2" t="inlineStr">
+        <is>
+          <t>distributor_authorization</t>
+        </is>
+      </c>
+      <c r="M2" s="2" t="inlineStr">
+        <is>
           <t>default_currency</t>
         </is>
       </c>
@@ -598,6 +618,21 @@
       </c>
       <c r="J3" s="3" t="inlineStr">
         <is>
+          <t>NET30</t>
+        </is>
+      </c>
+      <c r="K3" s="3" t="inlineStr">
+        <is>
+          <t>Distributor</t>
+        </is>
+      </c>
+      <c r="L3" s="3" t="inlineStr">
+        <is>
+          <t>Authorized Distributor</t>
+        </is>
+      </c>
+      <c r="M3" s="3" t="inlineStr">
+        <is>
           <t>USD</t>
         </is>
       </c>
@@ -650,6 +685,21 @@
       </c>
       <c r="J4" s="4" t="inlineStr">
         <is>
+          <t>NET45</t>
+        </is>
+      </c>
+      <c r="K4" s="4" t="inlineStr">
+        <is>
+          <t>Distributor</t>
+        </is>
+      </c>
+      <c r="L4" s="4" t="inlineStr">
+        <is>
+          <t>Authorized Distributor</t>
+        </is>
+      </c>
+      <c r="M4" s="4" t="inlineStr">
+        <is>
           <t>USD</t>
         </is>
       </c>
@@ -702,6 +752,21 @@
       </c>
       <c r="J5" s="3" t="inlineStr">
         <is>
+          <t>NET30</t>
+        </is>
+      </c>
+      <c r="K5" s="3" t="inlineStr">
+        <is>
+          <t>Distributor</t>
+        </is>
+      </c>
+      <c r="L5" s="3" t="inlineStr">
+        <is>
+          <t>Authorized Distributor</t>
+        </is>
+      </c>
+      <c r="M5" s="3" t="inlineStr">
+        <is>
           <t>CAD</t>
         </is>
       </c>
@@ -754,6 +819,21 @@
       </c>
       <c r="J6" s="4" t="inlineStr">
         <is>
+          <t>NET60</t>
+        </is>
+      </c>
+      <c r="K6" s="4" t="inlineStr">
+        <is>
+          <t>Retailer</t>
+        </is>
+      </c>
+      <c r="L6" s="4" t="inlineStr">
+        <is>
+          <t>Non-Distributor</t>
+        </is>
+      </c>
+      <c r="M6" s="4" t="inlineStr">
+        <is>
           <t>USD</t>
         </is>
       </c>
@@ -806,6 +886,21 @@
       </c>
       <c r="J7" s="3" t="inlineStr">
         <is>
+          <t>PREPAYMENT</t>
+        </is>
+      </c>
+      <c r="K7" s="3" t="inlineStr">
+        <is>
+          <t>Contractor</t>
+        </is>
+      </c>
+      <c r="L7" s="3" t="inlineStr">
+        <is>
+          <t>Non-Distributor</t>
+        </is>
+      </c>
+      <c r="M7" s="3" t="inlineStr">
+        <is>
           <t>USD</t>
         </is>
       </c>
@@ -858,19 +953,2353 @@
       </c>
       <c r="J8" s="4" t="inlineStr">
         <is>
+          <t>PREPAYMENT</t>
+        </is>
+      </c>
+      <c r="K8" s="4" t="inlineStr">
+        <is>
+          <t>Contractor</t>
+        </is>
+      </c>
+      <c r="L8" s="4" t="inlineStr">
+        <is>
+          <t>Non-Distributor</t>
+        </is>
+      </c>
+      <c r="M8" s="4" t="inlineStr">
+        <is>
           <t>USD</t>
         </is>
       </c>
     </row>
   </sheetData>
   <mergeCells count="1">
-    <mergeCell ref="A1:J1"/>
+    <mergeCell ref="A1:M1"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:G25"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="18" customWidth="1" min="1" max="1"/>
+    <col width="18" customWidth="1" min="2" max="2"/>
+    <col width="16" customWidth="1" min="3" max="3"/>
+    <col width="14" customWidth="1" min="4" max="4"/>
+    <col width="16" customWidth="1" min="5" max="5"/>
+    <col width="14" customWidth="1" min="6" max="6"/>
+    <col width="10" customWidth="1" min="7" max="7"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="26" customHeight="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>ORDER HISTORY  (past orders — header; source for buying-history derivation)</t>
+        </is>
+      </c>
+    </row>
+    <row r="2" ht="22" customHeight="1">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>order_id</t>
+        </is>
+      </c>
+      <c r="B2" s="2" t="inlineStr">
+        <is>
+          <t>customer_account</t>
+        </is>
+      </c>
+      <c r="C2" s="2" t="inlineStr">
+        <is>
+          <t>po_number</t>
+        </is>
+      </c>
+      <c r="D2" s="2" t="inlineStr">
+        <is>
+          <t>order_date</t>
+        </is>
+      </c>
+      <c r="E2" s="2" t="inlineStr">
+        <is>
+          <t>order_status</t>
+        </is>
+      </c>
+      <c r="F2" s="2" t="inlineStr">
+        <is>
+          <t>order_total</t>
+        </is>
+      </c>
+      <c r="G2" s="2" t="inlineStr">
+        <is>
+          <t>currency</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="3" t="inlineStr">
+        <is>
+          <t>ORD-1001-001</t>
+        </is>
+      </c>
+      <c r="B3" s="3" t="inlineStr">
+        <is>
+          <t>CUST-1001</t>
+        </is>
+      </c>
+      <c r="C3" s="3" t="inlineStr">
+        <is>
+          <t>USPO-24-3110</t>
+        </is>
+      </c>
+      <c r="D3" s="3" t="inlineStr">
+        <is>
+          <t>2024-09-15</t>
+        </is>
+      </c>
+      <c r="E3" s="3" t="inlineStr">
+        <is>
+          <t>auto-approved</t>
+        </is>
+      </c>
+      <c r="F3" s="3" t="n">
+        <v>6050</v>
+      </c>
+      <c r="G3" s="3" t="inlineStr">
+        <is>
+          <t>USD</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="4" t="inlineStr">
+        <is>
+          <t>ORD-1001-002</t>
+        </is>
+      </c>
+      <c r="B4" s="4" t="inlineStr">
+        <is>
+          <t>CUST-1001</t>
+        </is>
+      </c>
+      <c r="C4" s="4" t="inlineStr">
+        <is>
+          <t>USPO-25-3204</t>
+        </is>
+      </c>
+      <c r="D4" s="4" t="inlineStr">
+        <is>
+          <t>2025-01-20</t>
+        </is>
+      </c>
+      <c r="E4" s="4" t="inlineStr">
+        <is>
+          <t>auto-approved</t>
+        </is>
+      </c>
+      <c r="F4" s="4" t="n">
+        <v>10146.4</v>
+      </c>
+      <c r="G4" s="4" t="inlineStr">
+        <is>
+          <t>USD</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="3" t="inlineStr">
+        <is>
+          <t>ORD-1001-003</t>
+        </is>
+      </c>
+      <c r="B5" s="3" t="inlineStr">
+        <is>
+          <t>CUST-1001</t>
+        </is>
+      </c>
+      <c r="C5" s="3" t="inlineStr">
+        <is>
+          <t>USPO-25-3388</t>
+        </is>
+      </c>
+      <c r="D5" s="3" t="inlineStr">
+        <is>
+          <t>2025-05-12</t>
+        </is>
+      </c>
+      <c r="E5" s="3" t="inlineStr">
+        <is>
+          <t>approved</t>
+        </is>
+      </c>
+      <c r="F5" s="3" t="n">
+        <v>5225</v>
+      </c>
+      <c r="G5" s="3" t="inlineStr">
+        <is>
+          <t>USD</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="4" t="inlineStr">
+        <is>
+          <t>ORD-1001-004</t>
+        </is>
+      </c>
+      <c r="B6" s="4" t="inlineStr">
+        <is>
+          <t>CUST-1001</t>
+        </is>
+      </c>
+      <c r="C6" s="4" t="inlineStr">
+        <is>
+          <t>USPO-25-3512</t>
+        </is>
+      </c>
+      <c r="D6" s="4" t="inlineStr">
+        <is>
+          <t>2025-09-08</t>
+        </is>
+      </c>
+      <c r="E6" s="4" t="inlineStr">
+        <is>
+          <t>auto-approved</t>
+        </is>
+      </c>
+      <c r="F6" s="4" t="n">
+        <v>9495.200000000001</v>
+      </c>
+      <c r="G6" s="4" t="inlineStr">
+        <is>
+          <t>USD</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="3" t="inlineStr">
+        <is>
+          <t>ORD-1001-005</t>
+        </is>
+      </c>
+      <c r="B7" s="3" t="inlineStr">
+        <is>
+          <t>CUST-1001</t>
+        </is>
+      </c>
+      <c r="C7" s="3" t="inlineStr">
+        <is>
+          <t>USPO-26-3640</t>
+        </is>
+      </c>
+      <c r="D7" s="3" t="inlineStr">
+        <is>
+          <t>2026-02-18</t>
+        </is>
+      </c>
+      <c r="E7" s="3" t="inlineStr">
+        <is>
+          <t>auto-approved</t>
+        </is>
+      </c>
+      <c r="F7" s="3" t="n">
+        <v>8800</v>
+      </c>
+      <c r="G7" s="3" t="inlineStr">
+        <is>
+          <t>USD</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="4" t="inlineStr">
+        <is>
+          <t>ORD-1001-006</t>
+        </is>
+      </c>
+      <c r="B8" s="4" t="inlineStr">
+        <is>
+          <t>CUST-1001</t>
+        </is>
+      </c>
+      <c r="C8" s="4" t="inlineStr">
+        <is>
+          <t>USPO-26-3781</t>
+        </is>
+      </c>
+      <c r="D8" s="4" t="inlineStr">
+        <is>
+          <t>2026-06-20</t>
+        </is>
+      </c>
+      <c r="E8" s="4" t="inlineStr">
+        <is>
+          <t>auto-approved</t>
+        </is>
+      </c>
+      <c r="F8" s="4" t="n">
+        <v>8047.6</v>
+      </c>
+      <c r="G8" s="4" t="inlineStr">
+        <is>
+          <t>USD</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="3" t="inlineStr">
+        <is>
+          <t>ORD-1002-001</t>
+        </is>
+      </c>
+      <c r="B9" s="3" t="inlineStr">
+        <is>
+          <t>CUST-1002</t>
+        </is>
+      </c>
+      <c r="C9" s="3" t="inlineStr">
+        <is>
+          <t>USPO-24-4102</t>
+        </is>
+      </c>
+      <c r="D9" s="3" t="inlineStr">
+        <is>
+          <t>2024-11-10</t>
+        </is>
+      </c>
+      <c r="E9" s="3" t="inlineStr">
+        <is>
+          <t>auto-approved</t>
+        </is>
+      </c>
+      <c r="F9" s="3" t="n">
+        <v>6118</v>
+      </c>
+      <c r="G9" s="3" t="inlineStr">
+        <is>
+          <t>USD</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="4" t="inlineStr">
+        <is>
+          <t>ORD-1002-002</t>
+        </is>
+      </c>
+      <c r="B10" s="4" t="inlineStr">
+        <is>
+          <t>CUST-1002</t>
+        </is>
+      </c>
+      <c r="C10" s="4" t="inlineStr">
+        <is>
+          <t>USPO-25-4231</t>
+        </is>
+      </c>
+      <c r="D10" s="4" t="inlineStr">
+        <is>
+          <t>2025-04-22</t>
+        </is>
+      </c>
+      <c r="E10" s="4" t="inlineStr">
+        <is>
+          <t>approved</t>
+        </is>
+      </c>
+      <c r="F10" s="4" t="n">
+        <v>6210</v>
+      </c>
+      <c r="G10" s="4" t="inlineStr">
+        <is>
+          <t>USD</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="3" t="inlineStr">
+        <is>
+          <t>ORD-1002-003</t>
+        </is>
+      </c>
+      <c r="B11" s="3" t="inlineStr">
+        <is>
+          <t>CUST-1002</t>
+        </is>
+      </c>
+      <c r="C11" s="3" t="inlineStr">
+        <is>
+          <t>USPO-25-4390</t>
+        </is>
+      </c>
+      <c r="D11" s="3" t="inlineStr">
+        <is>
+          <t>2025-10-05</t>
+        </is>
+      </c>
+      <c r="E11" s="3" t="inlineStr">
+        <is>
+          <t>auto-approved</t>
+        </is>
+      </c>
+      <c r="F11" s="3" t="n">
+        <v>5175</v>
+      </c>
+      <c r="G11" s="3" t="inlineStr">
+        <is>
+          <t>USD</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="4" t="inlineStr">
+        <is>
+          <t>ORD-1002-004</t>
+        </is>
+      </c>
+      <c r="B12" s="4" t="inlineStr">
+        <is>
+          <t>CUST-1002</t>
+        </is>
+      </c>
+      <c r="C12" s="4" t="inlineStr">
+        <is>
+          <t>USPO-26-4488</t>
+        </is>
+      </c>
+      <c r="D12" s="4" t="inlineStr">
+        <is>
+          <t>2026-03-14</t>
+        </is>
+      </c>
+      <c r="E12" s="4" t="inlineStr">
+        <is>
+          <t>auto-approved</t>
+        </is>
+      </c>
+      <c r="F12" s="4" t="n">
+        <v>5382</v>
+      </c>
+      <c r="G12" s="4" t="inlineStr">
+        <is>
+          <t>USD</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="3" t="inlineStr">
+        <is>
+          <t>ORD-1002-005</t>
+        </is>
+      </c>
+      <c r="B13" s="3" t="inlineStr">
+        <is>
+          <t>CUST-1002</t>
+        </is>
+      </c>
+      <c r="C13" s="3" t="inlineStr">
+        <is>
+          <t>USPO-26-4602</t>
+        </is>
+      </c>
+      <c r="D13" s="3" t="inlineStr">
+        <is>
+          <t>2026-05-28</t>
+        </is>
+      </c>
+      <c r="E13" s="3" t="inlineStr">
+        <is>
+          <t>auto-approved</t>
+        </is>
+      </c>
+      <c r="F13" s="3" t="n">
+        <v>4646</v>
+      </c>
+      <c r="G13" s="3" t="inlineStr">
+        <is>
+          <t>USD</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="4" t="inlineStr">
+        <is>
+          <t>ORD-2001-001</t>
+        </is>
+      </c>
+      <c r="B14" s="4" t="inlineStr">
+        <is>
+          <t>CUST-2001</t>
+        </is>
+      </c>
+      <c r="C14" s="4" t="inlineStr">
+        <is>
+          <t>CAPO-24-5101</t>
+        </is>
+      </c>
+      <c r="D14" s="4" t="inlineStr">
+        <is>
+          <t>2024-12-01</t>
+        </is>
+      </c>
+      <c r="E14" s="4" t="inlineStr">
+        <is>
+          <t>auto-approved</t>
+        </is>
+      </c>
+      <c r="F14" s="4" t="n">
+        <v>7157.6</v>
+      </c>
+      <c r="G14" s="4" t="inlineStr">
+        <is>
+          <t>CAD</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="3" t="inlineStr">
+        <is>
+          <t>ORD-2001-002</t>
+        </is>
+      </c>
+      <c r="B15" s="3" t="inlineStr">
+        <is>
+          <t>CUST-2001</t>
+        </is>
+      </c>
+      <c r="C15" s="3" t="inlineStr">
+        <is>
+          <t>CAPO-25-5230</t>
+        </is>
+      </c>
+      <c r="D15" s="3" t="inlineStr">
+        <is>
+          <t>2025-06-15</t>
+        </is>
+      </c>
+      <c r="E15" s="3" t="inlineStr">
+        <is>
+          <t>approved</t>
+        </is>
+      </c>
+      <c r="F15" s="3" t="n">
+        <v>6072</v>
+      </c>
+      <c r="G15" s="3" t="inlineStr">
+        <is>
+          <t>CAD</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="4" t="inlineStr">
+        <is>
+          <t>ORD-2001-003</t>
+        </is>
+      </c>
+      <c r="B16" s="4" t="inlineStr">
+        <is>
+          <t>CUST-2001</t>
+        </is>
+      </c>
+      <c r="C16" s="4" t="inlineStr">
+        <is>
+          <t>CAPO-25-5377</t>
+        </is>
+      </c>
+      <c r="D16" s="4" t="inlineStr">
+        <is>
+          <t>2025-11-20</t>
+        </is>
+      </c>
+      <c r="E16" s="4" t="inlineStr">
+        <is>
+          <t>auto-approved</t>
+        </is>
+      </c>
+      <c r="F16" s="4" t="n">
+        <v>5773</v>
+      </c>
+      <c r="G16" s="4" t="inlineStr">
+        <is>
+          <t>CAD</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="3" t="inlineStr">
+        <is>
+          <t>ORD-2001-004</t>
+        </is>
+      </c>
+      <c r="B17" s="3" t="inlineStr">
+        <is>
+          <t>CUST-2001</t>
+        </is>
+      </c>
+      <c r="C17" s="3" t="inlineStr">
+        <is>
+          <t>CAPO-26-5490</t>
+        </is>
+      </c>
+      <c r="D17" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-01</t>
+        </is>
+      </c>
+      <c r="E17" s="3" t="inlineStr">
+        <is>
+          <t>auto-approved</t>
+        </is>
+      </c>
+      <c r="F17" s="3" t="n">
+        <v>5262.4</v>
+      </c>
+      <c r="G17" s="3" t="inlineStr">
+        <is>
+          <t>CAD</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="4" t="inlineStr">
+        <is>
+          <t>ORD-5001-001</t>
+        </is>
+      </c>
+      <c r="B18" s="4" t="inlineStr">
+        <is>
+          <t>CUST-5001</t>
+        </is>
+      </c>
+      <c r="C18" s="4" t="inlineStr">
+        <is>
+          <t>USPO-25-6110</t>
+        </is>
+      </c>
+      <c r="D18" s="4" t="inlineStr">
+        <is>
+          <t>2025-03-10</t>
+        </is>
+      </c>
+      <c r="E18" s="4" t="inlineStr">
+        <is>
+          <t>approved</t>
+        </is>
+      </c>
+      <c r="F18" s="4" t="n">
+        <v>717.9</v>
+      </c>
+      <c r="G18" s="4" t="inlineStr">
+        <is>
+          <t>USD</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="3" t="inlineStr">
+        <is>
+          <t>ORD-5001-002</t>
+        </is>
+      </c>
+      <c r="B19" s="3" t="inlineStr">
+        <is>
+          <t>CUST-5001</t>
+        </is>
+      </c>
+      <c r="C19" s="3" t="inlineStr">
+        <is>
+          <t>USPO-25-6244</t>
+        </is>
+      </c>
+      <c r="D19" s="3" t="inlineStr">
+        <is>
+          <t>2025-08-18</t>
+        </is>
+      </c>
+      <c r="E19" s="3" t="inlineStr">
+        <is>
+          <t>auto-approved</t>
+        </is>
+      </c>
+      <c r="F19" s="3" t="n">
+        <v>5626</v>
+      </c>
+      <c r="G19" s="3" t="inlineStr">
+        <is>
+          <t>USD</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="4" t="inlineStr">
+        <is>
+          <t>ORD-5001-003</t>
+        </is>
+      </c>
+      <c r="B20" s="4" t="inlineStr">
+        <is>
+          <t>CUST-5001</t>
+        </is>
+      </c>
+      <c r="C20" s="4" t="inlineStr">
+        <is>
+          <t>USPO-26-6351</t>
+        </is>
+      </c>
+      <c r="D20" s="4" t="inlineStr">
+        <is>
+          <t>2026-01-25</t>
+        </is>
+      </c>
+      <c r="E20" s="4" t="inlineStr">
+        <is>
+          <t>auto-approved</t>
+        </is>
+      </c>
+      <c r="F20" s="4" t="n">
+        <v>567.6</v>
+      </c>
+      <c r="G20" s="4" t="inlineStr">
+        <is>
+          <t>USD</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="3" t="inlineStr">
+        <is>
+          <t>ORD-5001-004</t>
+        </is>
+      </c>
+      <c r="B21" s="3" t="inlineStr">
+        <is>
+          <t>CUST-5001</t>
+        </is>
+      </c>
+      <c r="C21" s="3" t="inlineStr">
+        <is>
+          <t>USPO-26-6470</t>
+        </is>
+      </c>
+      <c r="D21" s="3" t="inlineStr">
+        <is>
+          <t>2026-04-15</t>
+        </is>
+      </c>
+      <c r="E21" s="3" t="inlineStr">
+        <is>
+          <t>approved</t>
+        </is>
+      </c>
+      <c r="F21" s="3" t="n">
+        <v>4626.9</v>
+      </c>
+      <c r="G21" s="3" t="inlineStr">
+        <is>
+          <t>USD</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="4" t="inlineStr">
+        <is>
+          <t>ORD-7000-001</t>
+        </is>
+      </c>
+      <c r="B22" s="4" t="inlineStr">
+        <is>
+          <t>CUST-7000</t>
+        </is>
+      </c>
+      <c r="C22" s="4" t="inlineStr">
+        <is>
+          <t>USPO-24-7101</t>
+        </is>
+      </c>
+      <c r="D22" s="4" t="inlineStr">
+        <is>
+          <t>2024-07-12</t>
+        </is>
+      </c>
+      <c r="E22" s="4" t="inlineStr">
+        <is>
+          <t>approved</t>
+        </is>
+      </c>
+      <c r="F22" s="4" t="n">
+        <v>6183</v>
+      </c>
+      <c r="G22" s="4" t="inlineStr">
+        <is>
+          <t>USD</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="3" t="inlineStr">
+        <is>
+          <t>ORD-7000-002</t>
+        </is>
+      </c>
+      <c r="B23" s="3" t="inlineStr">
+        <is>
+          <t>CUST-7000</t>
+        </is>
+      </c>
+      <c r="C23" s="3" t="inlineStr">
+        <is>
+          <t>USPO-25-7230</t>
+        </is>
+      </c>
+      <c r="D23" s="3" t="inlineStr">
+        <is>
+          <t>2025-02-08</t>
+        </is>
+      </c>
+      <c r="E23" s="3" t="inlineStr">
+        <is>
+          <t>approved</t>
+        </is>
+      </c>
+      <c r="F23" s="3" t="n">
+        <v>3492</v>
+      </c>
+      <c r="G23" s="3" t="inlineStr">
+        <is>
+          <t>USD</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="4" t="inlineStr">
+        <is>
+          <t>ORD-7000-003</t>
+        </is>
+      </c>
+      <c r="B24" s="4" t="inlineStr">
+        <is>
+          <t>CUST-7000</t>
+        </is>
+      </c>
+      <c r="C24" s="4" t="inlineStr">
+        <is>
+          <t>USPO-25-7388</t>
+        </is>
+      </c>
+      <c r="D24" s="4" t="inlineStr">
+        <is>
+          <t>2025-08-30</t>
+        </is>
+      </c>
+      <c r="E24" s="4" t="inlineStr">
+        <is>
+          <t>on-hold</t>
+        </is>
+      </c>
+      <c r="F24" s="4" t="n">
+        <v>5382.9</v>
+      </c>
+      <c r="G24" s="4" t="inlineStr">
+        <is>
+          <t>USD</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="3" t="inlineStr">
+        <is>
+          <t>ORD-7000-004</t>
+        </is>
+      </c>
+      <c r="B25" s="3" t="inlineStr">
+        <is>
+          <t>CUST-7000</t>
+        </is>
+      </c>
+      <c r="C25" s="3" t="inlineStr">
+        <is>
+          <t>USPO-26-7455</t>
+        </is>
+      </c>
+      <c r="D25" s="3" t="inlineStr">
+        <is>
+          <t>2026-03-10</t>
+        </is>
+      </c>
+      <c r="E25" s="3" t="inlineStr">
+        <is>
+          <t>on-hold</t>
+        </is>
+      </c>
+      <c r="F25" s="3" t="n">
+        <v>3055.5</v>
+      </c>
+      <c r="G25" s="3" t="inlineStr">
+        <is>
+          <t>USD</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="1">
+    <mergeCell ref="A1:G1"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:H40"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="22" customWidth="1" min="1" max="1"/>
+    <col width="18" customWidth="1" min="2" max="2"/>
+    <col width="16" customWidth="1" min="3" max="3"/>
+    <col width="16" customWidth="1" min="4" max="4"/>
+    <col width="12" customWidth="1" min="5" max="5"/>
+    <col width="10" customWidth="1" min="6" max="6"/>
+    <col width="12" customWidth="1" min="7" max="7"/>
+    <col width="14" customWidth="1" min="8" max="8"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="26" customHeight="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>ORDER HISTORY LINES  (past order line items — SKU / qty / price detail)</t>
+        </is>
+      </c>
+    </row>
+    <row r="2" ht="22" customHeight="1">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>order_line_id</t>
+        </is>
+      </c>
+      <c r="B2" s="2" t="inlineStr">
+        <is>
+          <t>order_id</t>
+        </is>
+      </c>
+      <c r="C2" s="2" t="inlineStr">
+        <is>
+          <t>sku</t>
+        </is>
+      </c>
+      <c r="D2" s="2" t="inlineStr">
+        <is>
+          <t>product_family</t>
+        </is>
+      </c>
+      <c r="E2" s="2" t="inlineStr">
+        <is>
+          <t>quantity</t>
+        </is>
+      </c>
+      <c r="F2" s="2" t="inlineStr">
+        <is>
+          <t>uom</t>
+        </is>
+      </c>
+      <c r="G2" s="2" t="inlineStr">
+        <is>
+          <t>unit_price</t>
+        </is>
+      </c>
+      <c r="H2" s="2" t="inlineStr">
+        <is>
+          <t>line_total</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="3" t="inlineStr">
+        <is>
+          <t>OL-ORD-1001-001-1</t>
+        </is>
+      </c>
+      <c r="B3" s="3" t="inlineStr">
+        <is>
+          <t>ORD-1001-001</t>
+        </is>
+      </c>
+      <c r="C3" s="3" t="inlineStr">
+        <is>
+          <t>SKU-CTG-4520</t>
+        </is>
+      </c>
+      <c r="D3" s="3" t="inlineStr">
+        <is>
+          <t>CARTRIDGE</t>
+        </is>
+      </c>
+      <c r="E3" s="3" t="n">
+        <v>400</v>
+      </c>
+      <c r="F3" s="3" t="inlineStr">
+        <is>
+          <t>EA</t>
+        </is>
+      </c>
+      <c r="G3" s="3" t="n">
+        <v>11</v>
+      </c>
+      <c r="H3" s="3" t="n">
+        <v>4400</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="4" t="inlineStr">
+        <is>
+          <t>OL-ORD-1001-001-2</t>
+        </is>
+      </c>
+      <c r="B4" s="4" t="inlineStr">
+        <is>
+          <t>ORD-1001-001</t>
+        </is>
+      </c>
+      <c r="C4" s="4" t="inlineStr">
+        <is>
+          <t>SKU-SEL-1150</t>
+        </is>
+      </c>
+      <c r="D4" s="4" t="inlineStr">
+        <is>
+          <t>SEAL</t>
+        </is>
+      </c>
+      <c r="E4" s="4" t="n">
+        <v>300</v>
+      </c>
+      <c r="F4" s="4" t="inlineStr">
+        <is>
+          <t>EA</t>
+        </is>
+      </c>
+      <c r="G4" s="4" t="n">
+        <v>5.5</v>
+      </c>
+      <c r="H4" s="4" t="n">
+        <v>1650</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="3" t="inlineStr">
+        <is>
+          <t>OL-ORD-1001-002-1</t>
+        </is>
+      </c>
+      <c r="B5" s="3" t="inlineStr">
+        <is>
+          <t>ORD-1001-002</t>
+        </is>
+      </c>
+      <c r="C5" s="3" t="inlineStr">
+        <is>
+          <t>SKU-CTG-4520</t>
+        </is>
+      </c>
+      <c r="D5" s="3" t="inlineStr">
+        <is>
+          <t>CARTRIDGE</t>
+        </is>
+      </c>
+      <c r="E5" s="3" t="n">
+        <v>500</v>
+      </c>
+      <c r="F5" s="3" t="inlineStr">
+        <is>
+          <t>EA</t>
+        </is>
+      </c>
+      <c r="G5" s="3" t="n">
+        <v>11</v>
+      </c>
+      <c r="H5" s="3" t="n">
+        <v>5500</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="4" t="inlineStr">
+        <is>
+          <t>OL-ORD-1001-002-2</t>
+        </is>
+      </c>
+      <c r="B6" s="4" t="inlineStr">
+        <is>
+          <t>ORD-1001-002</t>
+        </is>
+      </c>
+      <c r="C6" s="4" t="inlineStr">
+        <is>
+          <t>SKU-VLV-2201</t>
+        </is>
+      </c>
+      <c r="D6" s="4" t="inlineStr">
+        <is>
+          <t>VALVE</t>
+        </is>
+      </c>
+      <c r="E6" s="4" t="n">
+        <v>60</v>
+      </c>
+      <c r="F6" s="4" t="inlineStr">
+        <is>
+          <t>EA</t>
+        </is>
+      </c>
+      <c r="G6" s="4" t="n">
+        <v>77.44</v>
+      </c>
+      <c r="H6" s="4" t="n">
+        <v>4646.4</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="3" t="inlineStr">
+        <is>
+          <t>OL-ORD-1001-003-1</t>
+        </is>
+      </c>
+      <c r="B7" s="3" t="inlineStr">
+        <is>
+          <t>ORD-1001-003</t>
+        </is>
+      </c>
+      <c r="C7" s="3" t="inlineStr">
+        <is>
+          <t>SKU-CTG-4520</t>
+        </is>
+      </c>
+      <c r="D7" s="3" t="inlineStr">
+        <is>
+          <t>CARTRIDGE</t>
+        </is>
+      </c>
+      <c r="E7" s="3" t="n">
+        <v>350</v>
+      </c>
+      <c r="F7" s="3" t="inlineStr">
+        <is>
+          <t>EA</t>
+        </is>
+      </c>
+      <c r="G7" s="3" t="n">
+        <v>11</v>
+      </c>
+      <c r="H7" s="3" t="n">
+        <v>3850</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="4" t="inlineStr">
+        <is>
+          <t>OL-ORD-1001-003-2</t>
+        </is>
+      </c>
+      <c r="B8" s="4" t="inlineStr">
+        <is>
+          <t>ORD-1001-003</t>
+        </is>
+      </c>
+      <c r="C8" s="4" t="inlineStr">
+        <is>
+          <t>SKU-SEL-1150</t>
+        </is>
+      </c>
+      <c r="D8" s="4" t="inlineStr">
+        <is>
+          <t>SEAL</t>
+        </is>
+      </c>
+      <c r="E8" s="4" t="n">
+        <v>250</v>
+      </c>
+      <c r="F8" s="4" t="inlineStr">
+        <is>
+          <t>EA</t>
+        </is>
+      </c>
+      <c r="G8" s="4" t="n">
+        <v>5.5</v>
+      </c>
+      <c r="H8" s="4" t="n">
+        <v>1375</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="3" t="inlineStr">
+        <is>
+          <t>OL-ORD-1001-004-1</t>
+        </is>
+      </c>
+      <c r="B9" s="3" t="inlineStr">
+        <is>
+          <t>ORD-1001-004</t>
+        </is>
+      </c>
+      <c r="C9" s="3" t="inlineStr">
+        <is>
+          <t>SKU-VLV-2201</t>
+        </is>
+      </c>
+      <c r="D9" s="3" t="inlineStr">
+        <is>
+          <t>VALVE</t>
+        </is>
+      </c>
+      <c r="E9" s="3" t="n">
+        <v>80</v>
+      </c>
+      <c r="F9" s="3" t="inlineStr">
+        <is>
+          <t>EA</t>
+        </is>
+      </c>
+      <c r="G9" s="3" t="n">
+        <v>77.44</v>
+      </c>
+      <c r="H9" s="3" t="n">
+        <v>6195.2</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="4" t="inlineStr">
+        <is>
+          <t>OL-ORD-1001-004-2</t>
+        </is>
+      </c>
+      <c r="B10" s="4" t="inlineStr">
+        <is>
+          <t>ORD-1001-004</t>
+        </is>
+      </c>
+      <c r="C10" s="4" t="inlineStr">
+        <is>
+          <t>SKU-CTG-4520</t>
+        </is>
+      </c>
+      <c r="D10" s="4" t="inlineStr">
+        <is>
+          <t>CARTRIDGE</t>
+        </is>
+      </c>
+      <c r="E10" s="4" t="n">
+        <v>300</v>
+      </c>
+      <c r="F10" s="4" t="inlineStr">
+        <is>
+          <t>EA</t>
+        </is>
+      </c>
+      <c r="G10" s="4" t="n">
+        <v>11</v>
+      </c>
+      <c r="H10" s="4" t="n">
+        <v>3300</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="3" t="inlineStr">
+        <is>
+          <t>OL-ORD-1001-005-1</t>
+        </is>
+      </c>
+      <c r="B11" s="3" t="inlineStr">
+        <is>
+          <t>ORD-1001-005</t>
+        </is>
+      </c>
+      <c r="C11" s="3" t="inlineStr">
+        <is>
+          <t>SKU-CTG-4520</t>
+        </is>
+      </c>
+      <c r="D11" s="3" t="inlineStr">
+        <is>
+          <t>CARTRIDGE</t>
+        </is>
+      </c>
+      <c r="E11" s="3" t="n">
+        <v>600</v>
+      </c>
+      <c r="F11" s="3" t="inlineStr">
+        <is>
+          <t>EA</t>
+        </is>
+      </c>
+      <c r="G11" s="3" t="n">
+        <v>11</v>
+      </c>
+      <c r="H11" s="3" t="n">
+        <v>6600</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="4" t="inlineStr">
+        <is>
+          <t>OL-ORD-1001-005-2</t>
+        </is>
+      </c>
+      <c r="B12" s="4" t="inlineStr">
+        <is>
+          <t>ORD-1001-005</t>
+        </is>
+      </c>
+      <c r="C12" s="4" t="inlineStr">
+        <is>
+          <t>SKU-SEL-1150</t>
+        </is>
+      </c>
+      <c r="D12" s="4" t="inlineStr">
+        <is>
+          <t>SEAL</t>
+        </is>
+      </c>
+      <c r="E12" s="4" t="n">
+        <v>400</v>
+      </c>
+      <c r="F12" s="4" t="inlineStr">
+        <is>
+          <t>EA</t>
+        </is>
+      </c>
+      <c r="G12" s="4" t="n">
+        <v>5.5</v>
+      </c>
+      <c r="H12" s="4" t="n">
+        <v>2200</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="3" t="inlineStr">
+        <is>
+          <t>OL-ORD-1001-006-1</t>
+        </is>
+      </c>
+      <c r="B13" s="3" t="inlineStr">
+        <is>
+          <t>ORD-1001-006</t>
+        </is>
+      </c>
+      <c r="C13" s="3" t="inlineStr">
+        <is>
+          <t>SKU-CTG-4520</t>
+        </is>
+      </c>
+      <c r="D13" s="3" t="inlineStr">
+        <is>
+          <t>CARTRIDGE</t>
+        </is>
+      </c>
+      <c r="E13" s="3" t="n">
+        <v>450</v>
+      </c>
+      <c r="F13" s="3" t="inlineStr">
+        <is>
+          <t>EA</t>
+        </is>
+      </c>
+      <c r="G13" s="3" t="n">
+        <v>11</v>
+      </c>
+      <c r="H13" s="3" t="n">
+        <v>4950</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="4" t="inlineStr">
+        <is>
+          <t>OL-ORD-1001-006-2</t>
+        </is>
+      </c>
+      <c r="B14" s="4" t="inlineStr">
+        <is>
+          <t>ORD-1001-006</t>
+        </is>
+      </c>
+      <c r="C14" s="4" t="inlineStr">
+        <is>
+          <t>SKU-VLV-2201</t>
+        </is>
+      </c>
+      <c r="D14" s="4" t="inlineStr">
+        <is>
+          <t>VALVE</t>
+        </is>
+      </c>
+      <c r="E14" s="4" t="n">
+        <v>40</v>
+      </c>
+      <c r="F14" s="4" t="inlineStr">
+        <is>
+          <t>EA</t>
+        </is>
+      </c>
+      <c r="G14" s="4" t="n">
+        <v>77.44</v>
+      </c>
+      <c r="H14" s="4" t="n">
+        <v>3097.6</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="3" t="inlineStr">
+        <is>
+          <t>OL-ORD-1002-001-1</t>
+        </is>
+      </c>
+      <c r="B15" s="3" t="inlineStr">
+        <is>
+          <t>ORD-1002-001</t>
+        </is>
+      </c>
+      <c r="C15" s="3" t="inlineStr">
+        <is>
+          <t>SKU-DRN-3010</t>
+        </is>
+      </c>
+      <c r="D15" s="3" t="inlineStr">
+        <is>
+          <t>DRAIN</t>
+        </is>
+      </c>
+      <c r="E15" s="3" t="n">
+        <v>120</v>
+      </c>
+      <c r="F15" s="3" t="inlineStr">
+        <is>
+          <t>EA</t>
+        </is>
+      </c>
+      <c r="G15" s="3" t="n">
+        <v>41.4</v>
+      </c>
+      <c r="H15" s="3" t="n">
+        <v>4968</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="4" t="inlineStr">
+        <is>
+          <t>OL-ORD-1002-001-2</t>
+        </is>
+      </c>
+      <c r="B16" s="4" t="inlineStr">
+        <is>
+          <t>ORD-1002-001</t>
+        </is>
+      </c>
+      <c r="C16" s="4" t="inlineStr">
+        <is>
+          <t>SKU-SEL-1150</t>
+        </is>
+      </c>
+      <c r="D16" s="4" t="inlineStr">
+        <is>
+          <t>SEAL</t>
+        </is>
+      </c>
+      <c r="E16" s="4" t="n">
+        <v>200</v>
+      </c>
+      <c r="F16" s="4" t="inlineStr">
+        <is>
+          <t>EA</t>
+        </is>
+      </c>
+      <c r="G16" s="4" t="n">
+        <v>5.75</v>
+      </c>
+      <c r="H16" s="4" t="n">
+        <v>1150</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="3" t="inlineStr">
+        <is>
+          <t>OL-ORD-1002-002-1</t>
+        </is>
+      </c>
+      <c r="B17" s="3" t="inlineStr">
+        <is>
+          <t>ORD-1002-002</t>
+        </is>
+      </c>
+      <c r="C17" s="3" t="inlineStr">
+        <is>
+          <t>SKU-DRN-3010</t>
+        </is>
+      </c>
+      <c r="D17" s="3" t="inlineStr">
+        <is>
+          <t>DRAIN</t>
+        </is>
+      </c>
+      <c r="E17" s="3" t="n">
+        <v>150</v>
+      </c>
+      <c r="F17" s="3" t="inlineStr">
+        <is>
+          <t>EA</t>
+        </is>
+      </c>
+      <c r="G17" s="3" t="n">
+        <v>41.4</v>
+      </c>
+      <c r="H17" s="3" t="n">
+        <v>6210</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="4" t="inlineStr">
+        <is>
+          <t>OL-ORD-1002-003-1</t>
+        </is>
+      </c>
+      <c r="B18" s="4" t="inlineStr">
+        <is>
+          <t>ORD-1002-003</t>
+        </is>
+      </c>
+      <c r="C18" s="4" t="inlineStr">
+        <is>
+          <t>SKU-DRN-3010</t>
+        </is>
+      </c>
+      <c r="D18" s="4" t="inlineStr">
+        <is>
+          <t>DRAIN</t>
+        </is>
+      </c>
+      <c r="E18" s="4" t="n">
+        <v>100</v>
+      </c>
+      <c r="F18" s="4" t="inlineStr">
+        <is>
+          <t>EA</t>
+        </is>
+      </c>
+      <c r="G18" s="4" t="n">
+        <v>41.4</v>
+      </c>
+      <c r="H18" s="4" t="n">
+        <v>4140</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="3" t="inlineStr">
+        <is>
+          <t>OL-ORD-1002-003-2</t>
+        </is>
+      </c>
+      <c r="B19" s="3" t="inlineStr">
+        <is>
+          <t>ORD-1002-003</t>
+        </is>
+      </c>
+      <c r="C19" s="3" t="inlineStr">
+        <is>
+          <t>SKU-SEL-1150</t>
+        </is>
+      </c>
+      <c r="D19" s="3" t="inlineStr">
+        <is>
+          <t>SEAL</t>
+        </is>
+      </c>
+      <c r="E19" s="3" t="n">
+        <v>180</v>
+      </c>
+      <c r="F19" s="3" t="inlineStr">
+        <is>
+          <t>EA</t>
+        </is>
+      </c>
+      <c r="G19" s="3" t="n">
+        <v>5.75</v>
+      </c>
+      <c r="H19" s="3" t="n">
+        <v>1035</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="4" t="inlineStr">
+        <is>
+          <t>OL-ORD-1002-004-1</t>
+        </is>
+      </c>
+      <c r="B20" s="4" t="inlineStr">
+        <is>
+          <t>ORD-1002-004</t>
+        </is>
+      </c>
+      <c r="C20" s="4" t="inlineStr">
+        <is>
+          <t>SKU-DRN-3010</t>
+        </is>
+      </c>
+      <c r="D20" s="4" t="inlineStr">
+        <is>
+          <t>DRAIN</t>
+        </is>
+      </c>
+      <c r="E20" s="4" t="n">
+        <v>130</v>
+      </c>
+      <c r="F20" s="4" t="inlineStr">
+        <is>
+          <t>EA</t>
+        </is>
+      </c>
+      <c r="G20" s="4" t="n">
+        <v>41.4</v>
+      </c>
+      <c r="H20" s="4" t="n">
+        <v>5382</v>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="3" t="inlineStr">
+        <is>
+          <t>OL-ORD-1002-005-1</t>
+        </is>
+      </c>
+      <c r="B21" s="3" t="inlineStr">
+        <is>
+          <t>ORD-1002-005</t>
+        </is>
+      </c>
+      <c r="C21" s="3" t="inlineStr">
+        <is>
+          <t>SKU-DRN-3010</t>
+        </is>
+      </c>
+      <c r="D21" s="3" t="inlineStr">
+        <is>
+          <t>DRAIN</t>
+        </is>
+      </c>
+      <c r="E21" s="3" t="n">
+        <v>90</v>
+      </c>
+      <c r="F21" s="3" t="inlineStr">
+        <is>
+          <t>EA</t>
+        </is>
+      </c>
+      <c r="G21" s="3" t="n">
+        <v>41.4</v>
+      </c>
+      <c r="H21" s="3" t="n">
+        <v>3726</v>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="4" t="inlineStr">
+        <is>
+          <t>OL-ORD-1002-005-2</t>
+        </is>
+      </c>
+      <c r="B22" s="4" t="inlineStr">
+        <is>
+          <t>ORD-1002-005</t>
+        </is>
+      </c>
+      <c r="C22" s="4" t="inlineStr">
+        <is>
+          <t>SKU-SEL-1150</t>
+        </is>
+      </c>
+      <c r="D22" s="4" t="inlineStr">
+        <is>
+          <t>SEAL</t>
+        </is>
+      </c>
+      <c r="E22" s="4" t="n">
+        <v>160</v>
+      </c>
+      <c r="F22" s="4" t="inlineStr">
+        <is>
+          <t>EA</t>
+        </is>
+      </c>
+      <c r="G22" s="4" t="n">
+        <v>5.75</v>
+      </c>
+      <c r="H22" s="4" t="n">
+        <v>920</v>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="3" t="inlineStr">
+        <is>
+          <t>OL-ORD-2001-001-1</t>
+        </is>
+      </c>
+      <c r="B23" s="3" t="inlineStr">
+        <is>
+          <t>ORD-2001-001</t>
+        </is>
+      </c>
+      <c r="C23" s="3" t="inlineStr">
+        <is>
+          <t>SKU-VLV-2201</t>
+        </is>
+      </c>
+      <c r="D23" s="3" t="inlineStr">
+        <is>
+          <t>VALVE</t>
+        </is>
+      </c>
+      <c r="E23" s="3" t="n">
+        <v>60</v>
+      </c>
+      <c r="F23" s="3" t="inlineStr">
+        <is>
+          <t>EA</t>
+        </is>
+      </c>
+      <c r="G23" s="3" t="n">
+        <v>80.95999999999999</v>
+      </c>
+      <c r="H23" s="3" t="n">
+        <v>4857.6</v>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="4" t="inlineStr">
+        <is>
+          <t>OL-ORD-2001-001-2</t>
+        </is>
+      </c>
+      <c r="B24" s="4" t="inlineStr">
+        <is>
+          <t>ORD-2001-001</t>
+        </is>
+      </c>
+      <c r="C24" s="4" t="inlineStr">
+        <is>
+          <t>SKU-CTG-4520</t>
+        </is>
+      </c>
+      <c r="D24" s="4" t="inlineStr">
+        <is>
+          <t>CARTRIDGE</t>
+        </is>
+      </c>
+      <c r="E24" s="4" t="n">
+        <v>200</v>
+      </c>
+      <c r="F24" s="4" t="inlineStr">
+        <is>
+          <t>EA</t>
+        </is>
+      </c>
+      <c r="G24" s="4" t="n">
+        <v>11.5</v>
+      </c>
+      <c r="H24" s="4" t="n">
+        <v>2300</v>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="3" t="inlineStr">
+        <is>
+          <t>OL-ORD-2001-002-1</t>
+        </is>
+      </c>
+      <c r="B25" s="3" t="inlineStr">
+        <is>
+          <t>ORD-2001-002</t>
+        </is>
+      </c>
+      <c r="C25" s="3" t="inlineStr">
+        <is>
+          <t>SKU-VLV-2201</t>
+        </is>
+      </c>
+      <c r="D25" s="3" t="inlineStr">
+        <is>
+          <t>VALVE</t>
+        </is>
+      </c>
+      <c r="E25" s="3" t="n">
+        <v>75</v>
+      </c>
+      <c r="F25" s="3" t="inlineStr">
+        <is>
+          <t>EA</t>
+        </is>
+      </c>
+      <c r="G25" s="3" t="n">
+        <v>80.95999999999999</v>
+      </c>
+      <c r="H25" s="3" t="n">
+        <v>6072</v>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="4" t="inlineStr">
+        <is>
+          <t>OL-ORD-2001-003-1</t>
+        </is>
+      </c>
+      <c r="B26" s="4" t="inlineStr">
+        <is>
+          <t>ORD-2001-003</t>
+        </is>
+      </c>
+      <c r="C26" s="4" t="inlineStr">
+        <is>
+          <t>SKU-VLV-2201</t>
+        </is>
+      </c>
+      <c r="D26" s="4" t="inlineStr">
+        <is>
+          <t>VALVE</t>
+        </is>
+      </c>
+      <c r="E26" s="4" t="n">
+        <v>50</v>
+      </c>
+      <c r="F26" s="4" t="inlineStr">
+        <is>
+          <t>EA</t>
+        </is>
+      </c>
+      <c r="G26" s="4" t="n">
+        <v>80.95999999999999</v>
+      </c>
+      <c r="H26" s="4" t="n">
+        <v>4048</v>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="3" t="inlineStr">
+        <is>
+          <t>OL-ORD-2001-003-2</t>
+        </is>
+      </c>
+      <c r="B27" s="3" t="inlineStr">
+        <is>
+          <t>ORD-2001-003</t>
+        </is>
+      </c>
+      <c r="C27" s="3" t="inlineStr">
+        <is>
+          <t>SKU-CTG-4520</t>
+        </is>
+      </c>
+      <c r="D27" s="3" t="inlineStr">
+        <is>
+          <t>CARTRIDGE</t>
+        </is>
+      </c>
+      <c r="E27" s="3" t="n">
+        <v>150</v>
+      </c>
+      <c r="F27" s="3" t="inlineStr">
+        <is>
+          <t>EA</t>
+        </is>
+      </c>
+      <c r="G27" s="3" t="n">
+        <v>11.5</v>
+      </c>
+      <c r="H27" s="3" t="n">
+        <v>1725</v>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="4" t="inlineStr">
+        <is>
+          <t>OL-ORD-2001-004-1</t>
+        </is>
+      </c>
+      <c r="B28" s="4" t="inlineStr">
+        <is>
+          <t>ORD-2001-004</t>
+        </is>
+      </c>
+      <c r="C28" s="4" t="inlineStr">
+        <is>
+          <t>SKU-VLV-2201</t>
+        </is>
+      </c>
+      <c r="D28" s="4" t="inlineStr">
+        <is>
+          <t>VALVE</t>
+        </is>
+      </c>
+      <c r="E28" s="4" t="n">
+        <v>65</v>
+      </c>
+      <c r="F28" s="4" t="inlineStr">
+        <is>
+          <t>EA</t>
+        </is>
+      </c>
+      <c r="G28" s="4" t="n">
+        <v>80.95999999999999</v>
+      </c>
+      <c r="H28" s="4" t="n">
+        <v>5262.4</v>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="3" t="inlineStr">
+        <is>
+          <t>OL-ORD-5001-001-1</t>
+        </is>
+      </c>
+      <c r="B29" s="3" t="inlineStr">
+        <is>
+          <t>ORD-5001-001</t>
+        </is>
+      </c>
+      <c r="C29" s="3" t="inlineStr">
+        <is>
+          <t>SKU-FIN-9100</t>
+        </is>
+      </c>
+      <c r="D29" s="3" t="inlineStr">
+        <is>
+          <t>FINISH</t>
+        </is>
+      </c>
+      <c r="E29" s="3" t="n">
+        <v>40</v>
+      </c>
+      <c r="F29" s="3" t="inlineStr">
+        <is>
+          <t>GAL</t>
+        </is>
+      </c>
+      <c r="G29" s="3" t="n">
+        <v>9.460000000000001</v>
+      </c>
+      <c r="H29" s="3" t="n">
+        <v>378.4</v>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="4" t="inlineStr">
+        <is>
+          <t>OL-ORD-5001-001-2</t>
+        </is>
+      </c>
+      <c r="B30" s="4" t="inlineStr">
+        <is>
+          <t>ORD-5001-001</t>
+        </is>
+      </c>
+      <c r="C30" s="4" t="inlineStr">
+        <is>
+          <t>SKU-FIN-9200</t>
+        </is>
+      </c>
+      <c r="D30" s="4" t="inlineStr">
+        <is>
+          <t>FINISH</t>
+        </is>
+      </c>
+      <c r="E30" s="4" t="n">
+        <v>25</v>
+      </c>
+      <c r="F30" s="4" t="inlineStr">
+        <is>
+          <t>GAL</t>
+        </is>
+      </c>
+      <c r="G30" s="4" t="n">
+        <v>13.58</v>
+      </c>
+      <c r="H30" s="4" t="n">
+        <v>339.5</v>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="3" t="inlineStr">
+        <is>
+          <t>OL-ORD-5001-002-1</t>
+        </is>
+      </c>
+      <c r="B31" s="3" t="inlineStr">
+        <is>
+          <t>ORD-5001-002</t>
+        </is>
+      </c>
+      <c r="C31" s="3" t="inlineStr">
+        <is>
+          <t>SKU-SHS-7700</t>
+        </is>
+      </c>
+      <c r="D31" s="3" t="inlineStr">
+        <is>
+          <t>SHOWERSYS</t>
+        </is>
+      </c>
+      <c r="E31" s="3" t="n">
+        <v>4</v>
+      </c>
+      <c r="F31" s="3" t="inlineStr">
+        <is>
+          <t>EA</t>
+        </is>
+      </c>
+      <c r="G31" s="3" t="n">
+        <v>1406.5</v>
+      </c>
+      <c r="H31" s="3" t="n">
+        <v>5626</v>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="4" t="inlineStr">
+        <is>
+          <t>OL-ORD-5001-003-1</t>
+        </is>
+      </c>
+      <c r="B32" s="4" t="inlineStr">
+        <is>
+          <t>ORD-5001-003</t>
+        </is>
+      </c>
+      <c r="C32" s="4" t="inlineStr">
+        <is>
+          <t>SKU-FIN-9100</t>
+        </is>
+      </c>
+      <c r="D32" s="4" t="inlineStr">
+        <is>
+          <t>FINISH</t>
+        </is>
+      </c>
+      <c r="E32" s="4" t="n">
+        <v>60</v>
+      </c>
+      <c r="F32" s="4" t="inlineStr">
+        <is>
+          <t>GAL</t>
+        </is>
+      </c>
+      <c r="G32" s="4" t="n">
+        <v>9.460000000000001</v>
+      </c>
+      <c r="H32" s="4" t="n">
+        <v>567.6</v>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="3" t="inlineStr">
+        <is>
+          <t>OL-ORD-5001-004-1</t>
+        </is>
+      </c>
+      <c r="B33" s="3" t="inlineStr">
+        <is>
+          <t>ORD-5001-004</t>
+        </is>
+      </c>
+      <c r="C33" s="3" t="inlineStr">
+        <is>
+          <t>SKU-SHS-7700</t>
+        </is>
+      </c>
+      <c r="D33" s="3" t="inlineStr">
+        <is>
+          <t>SHOWERSYS</t>
+        </is>
+      </c>
+      <c r="E33" s="3" t="n">
+        <v>3</v>
+      </c>
+      <c r="F33" s="3" t="inlineStr">
+        <is>
+          <t>EA</t>
+        </is>
+      </c>
+      <c r="G33" s="3" t="n">
+        <v>1406.5</v>
+      </c>
+      <c r="H33" s="3" t="n">
+        <v>4219.5</v>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="4" t="inlineStr">
+        <is>
+          <t>OL-ORD-5001-004-2</t>
+        </is>
+      </c>
+      <c r="B34" s="4" t="inlineStr">
+        <is>
+          <t>ORD-5001-004</t>
+        </is>
+      </c>
+      <c r="C34" s="4" t="inlineStr">
+        <is>
+          <t>SKU-FIN-9200</t>
+        </is>
+      </c>
+      <c r="D34" s="4" t="inlineStr">
+        <is>
+          <t>FINISH</t>
+        </is>
+      </c>
+      <c r="E34" s="4" t="n">
+        <v>30</v>
+      </c>
+      <c r="F34" s="4" t="inlineStr">
+        <is>
+          <t>GAL</t>
+        </is>
+      </c>
+      <c r="G34" s="4" t="n">
+        <v>13.58</v>
+      </c>
+      <c r="H34" s="4" t="n">
+        <v>407.4</v>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="3" t="inlineStr">
+        <is>
+          <t>OL-ORD-7000-001-1</t>
+        </is>
+      </c>
+      <c r="B35" s="3" t="inlineStr">
+        <is>
+          <t>ORD-7000-001</t>
+        </is>
+      </c>
+      <c r="C35" s="3" t="inlineStr">
+        <is>
+          <t>SKU-DRN-3010</t>
+        </is>
+      </c>
+      <c r="D35" s="3" t="inlineStr">
+        <is>
+          <t>DRAIN</t>
+        </is>
+      </c>
+      <c r="E35" s="3" t="n">
+        <v>100</v>
+      </c>
+      <c r="F35" s="3" t="inlineStr">
+        <is>
+          <t>EA</t>
+        </is>
+      </c>
+      <c r="G35" s="3" t="n">
+        <v>43.65</v>
+      </c>
+      <c r="H35" s="3" t="n">
+        <v>4365</v>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="4" t="inlineStr">
+        <is>
+          <t>OL-ORD-7000-001-2</t>
+        </is>
+      </c>
+      <c r="B36" s="4" t="inlineStr">
+        <is>
+          <t>ORD-7000-001</t>
+        </is>
+      </c>
+      <c r="C36" s="4" t="inlineStr">
+        <is>
+          <t>SKU-CTG-4520</t>
+        </is>
+      </c>
+      <c r="D36" s="4" t="inlineStr">
+        <is>
+          <t>CARTRIDGE</t>
+        </is>
+      </c>
+      <c r="E36" s="4" t="n">
+        <v>150</v>
+      </c>
+      <c r="F36" s="4" t="inlineStr">
+        <is>
+          <t>EA</t>
+        </is>
+      </c>
+      <c r="G36" s="4" t="n">
+        <v>12.12</v>
+      </c>
+      <c r="H36" s="4" t="n">
+        <v>1818</v>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="3" t="inlineStr">
+        <is>
+          <t>OL-ORD-7000-002-1</t>
+        </is>
+      </c>
+      <c r="B37" s="3" t="inlineStr">
+        <is>
+          <t>ORD-7000-002</t>
+        </is>
+      </c>
+      <c r="C37" s="3" t="inlineStr">
+        <is>
+          <t>SKU-DRN-3010</t>
+        </is>
+      </c>
+      <c r="D37" s="3" t="inlineStr">
+        <is>
+          <t>DRAIN</t>
+        </is>
+      </c>
+      <c r="E37" s="3" t="n">
+        <v>80</v>
+      </c>
+      <c r="F37" s="3" t="inlineStr">
+        <is>
+          <t>EA</t>
+        </is>
+      </c>
+      <c r="G37" s="3" t="n">
+        <v>43.65</v>
+      </c>
+      <c r="H37" s="3" t="n">
+        <v>3492</v>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="4" t="inlineStr">
+        <is>
+          <t>OL-ORD-7000-003-1</t>
+        </is>
+      </c>
+      <c r="B38" s="4" t="inlineStr">
+        <is>
+          <t>ORD-7000-003</t>
+        </is>
+      </c>
+      <c r="C38" s="4" t="inlineStr">
+        <is>
+          <t>SKU-CTG-4520</t>
+        </is>
+      </c>
+      <c r="D38" s="4" t="inlineStr">
+        <is>
+          <t>CARTRIDGE</t>
+        </is>
+      </c>
+      <c r="E38" s="4" t="n">
+        <v>120</v>
+      </c>
+      <c r="F38" s="4" t="inlineStr">
+        <is>
+          <t>EA</t>
+        </is>
+      </c>
+      <c r="G38" s="4" t="n">
+        <v>12.12</v>
+      </c>
+      <c r="H38" s="4" t="n">
+        <v>1454.4</v>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="3" t="inlineStr">
+        <is>
+          <t>OL-ORD-7000-003-2</t>
+        </is>
+      </c>
+      <c r="B39" s="3" t="inlineStr">
+        <is>
+          <t>ORD-7000-003</t>
+        </is>
+      </c>
+      <c r="C39" s="3" t="inlineStr">
+        <is>
+          <t>SKU-DRN-3010</t>
+        </is>
+      </c>
+      <c r="D39" s="3" t="inlineStr">
+        <is>
+          <t>DRAIN</t>
+        </is>
+      </c>
+      <c r="E39" s="3" t="n">
+        <v>90</v>
+      </c>
+      <c r="F39" s="3" t="inlineStr">
+        <is>
+          <t>EA</t>
+        </is>
+      </c>
+      <c r="G39" s="3" t="n">
+        <v>43.65</v>
+      </c>
+      <c r="H39" s="3" t="n">
+        <v>3928.5</v>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="4" t="inlineStr">
+        <is>
+          <t>OL-ORD-7000-004-1</t>
+        </is>
+      </c>
+      <c r="B40" s="4" t="inlineStr">
+        <is>
+          <t>ORD-7000-004</t>
+        </is>
+      </c>
+      <c r="C40" s="4" t="inlineStr">
+        <is>
+          <t>SKU-DRN-3010</t>
+        </is>
+      </c>
+      <c r="D40" s="4" t="inlineStr">
+        <is>
+          <t>DRAIN</t>
+        </is>
+      </c>
+      <c r="E40" s="4" t="n">
+        <v>70</v>
+      </c>
+      <c r="F40" s="4" t="inlineStr">
+        <is>
+          <t>EA</t>
+        </is>
+      </c>
+      <c r="G40" s="4" t="n">
+        <v>43.65</v>
+      </c>
+      <c r="H40" s="4" t="n">
+        <v>3055.5</v>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="1">
+    <mergeCell ref="A1:H1"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -1062,13 +3491,13 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N9"/>
+  <dimension ref="A1:O10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -1085,6 +3514,7 @@
     <col width="20" customWidth="1" min="12" max="12"/>
     <col width="18" customWidth="1" min="13" max="13"/>
     <col width="20" customWidth="1" min="14" max="14"/>
+    <col width="60" customWidth="1" min="15" max="15"/>
   </cols>
   <sheetData>
     <row r="1" ht="26" customHeight="1">
@@ -1165,6 +3595,11 @@
           <t>backorder_tolerance_days</t>
         </is>
       </c>
+      <c r="O2" s="2" t="inlineStr">
+        <is>
+          <t>default_delivery_instructions</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" s="3" t="inlineStr">
@@ -1235,6 +3670,11 @@
       <c r="N3" s="3" t="n">
         <v>0</v>
       </c>
+      <c r="O3" s="3" t="inlineStr">
+        <is>
+          <t>Deliver Mon-Fri 8am-4pm at DC receiving dock 3. Notify John Miller (312-555-0140) 30 min before arrival.</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" s="4" t="inlineStr">
@@ -1305,6 +3745,11 @@
       <c r="N4" s="4" t="n">
         <v>2</v>
       </c>
+      <c r="O4" s="4" t="inlineStr">
+        <is>
+          <t>Deliver Tue-Fri 9am-3pm at branch dock B. Call 313-555-0210 upon arrival.</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" s="3" t="inlineStr">
@@ -1375,6 +3820,11 @@
       <c r="N5" s="3" t="n">
         <v>3</v>
       </c>
+      <c r="O5" s="3" t="inlineStr">
+        <is>
+          <t>Delivery via freight elevator (rear entrance). Weekdays 7am-2pm only.</t>
+        </is>
+      </c>
     </row>
     <row r="6">
       <c r="A6" s="4" t="inlineStr">
@@ -1445,6 +3895,11 @@
       <c r="N6" s="4" t="n">
         <v>5</v>
       </c>
+      <c r="O6" s="4" t="inlineStr">
+        <is>
+          <t>Commercial delivery only. Provide customs documents in advance.</t>
+        </is>
+      </c>
     </row>
     <row r="7">
       <c r="A7" s="3" t="inlineStr">
@@ -1515,6 +3970,11 @@
       <c r="N7" s="3" t="n">
         <v>2</v>
       </c>
+      <c r="O7" s="3" t="inlineStr">
+        <is>
+          <t>Deliver 7am-3pm. Curbside drop only; no forklift on-site.</t>
+        </is>
+      </c>
     </row>
     <row r="8">
       <c r="A8" s="4" t="inlineStr">
@@ -1585,6 +4045,11 @@
       <c r="N8" s="4" t="n">
         <v>7</v>
       </c>
+      <c r="O8" s="4" t="inlineStr">
+        <is>
+          <t>Remote project site — coordinate with site supervisor 48 hours before arrival.</t>
+        </is>
+      </c>
     </row>
     <row r="9">
       <c r="A9" s="3" t="inlineStr">
@@ -1655,22 +4120,102 @@
       <c r="N9" s="3" t="n">
         <v>0</v>
       </c>
+      <c r="O9" s="3" t="inlineStr">
+        <is>
+          <t>White-glove delivery required. Do NOT leave unattended.</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="4" t="inlineStr">
+        <is>
+          <t>ST-CA-008</t>
+        </is>
+      </c>
+      <c r="B10" s="4" t="inlineStr">
+        <is>
+          <t>Great Lakes - Malibu Coast Project</t>
+        </is>
+      </c>
+      <c r="C10" s="4" t="inlineStr">
+        <is>
+          <t>22200 Pacific Coast Hwy, Malibu, CA</t>
+        </is>
+      </c>
+      <c r="D10" s="4" t="inlineStr">
+        <is>
+          <t>90265</t>
+        </is>
+      </c>
+      <c r="E10" s="4" t="inlineStr">
+        <is>
+          <t>BR-GLP-MW</t>
+        </is>
+      </c>
+      <c r="F10" s="4" t="inlineStr">
+        <is>
+          <t>ACTIVE</t>
+        </is>
+      </c>
+      <c r="G10" s="4" t="inlineStr">
+        <is>
+          <t>CUST-1001</t>
+        </is>
+      </c>
+      <c r="H10" s="4" t="inlineStr">
+        <is>
+          <t>Malibu</t>
+        </is>
+      </c>
+      <c r="I10" s="4" t="inlineStr">
+        <is>
+          <t>CA</t>
+        </is>
+      </c>
+      <c r="J10" s="4" t="inlineStr">
+        <is>
+          <t>US</t>
+        </is>
+      </c>
+      <c r="K10" s="4" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="L10" s="4" t="inlineStr">
+        <is>
+          <t>DC-LA-05</t>
+        </is>
+      </c>
+      <c r="M10" s="4" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="N10" s="4" t="n">
+        <v>3</v>
+      </c>
+      <c r="O10" s="4" t="inlineStr">
+        <is>
+          <t>Project site — access via service road. Contact foreman at 310-555-0090.</t>
+        </is>
+      </c>
     </row>
   </sheetData>
   <mergeCells count="1">
-    <mergeCell ref="A1:N1"/>
+    <mergeCell ref="A1:O1"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G17"/>
+  <dimension ref="A1:G18"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -2109,6 +4654,27 @@
         </is>
       </c>
     </row>
+    <row r="18">
+      <c r="A18" s="4" t="inlineStr">
+        <is>
+          <t>ship_to</t>
+        </is>
+      </c>
+      <c r="B18" s="4" t="inlineStr">
+        <is>
+          <t>ST-CA-008</t>
+        </is>
+      </c>
+      <c r="C18" s="4" t="inlineStr"/>
+      <c r="D18" s="4" t="inlineStr"/>
+      <c r="E18" s="4" t="inlineStr"/>
+      <c r="F18" s="4" t="inlineStr"/>
+      <c r="G18" s="4" t="inlineStr">
+        <is>
+          <t>RULE-COAST-TO-COAST</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <mergeCells count="1">
     <mergeCell ref="A1:G1"/>
@@ -2117,13 +4683,13 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L12"/>
+  <dimension ref="A1:L13"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -2552,7 +5118,7 @@
         <v>1</v>
       </c>
       <c r="J9" s="3" t="n">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="K9" s="3" t="inlineStr">
         <is>
@@ -2561,7 +5127,7 @@
       </c>
       <c r="L9" s="3" t="inlineStr">
         <is>
-          <t>Customer requires one shipment, no split, no backorder. Full quantity must come from a single DC or the order is held for CSR review.</t>
+          <t>Customer requires one shipment, no split, no backorder, within a tight 2-day delivery SLA. Full quantity must come from a single DC or the order is held for CSR review.</t>
         </is>
       </c>
     </row>
@@ -2722,6 +5288,58 @@
       <c r="L12" s="4" t="inlineStr">
         <is>
           <t>Bulk customer. Minimum total order quantity = 500 units. Smaller orders are rejected to protect margins.</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="3" t="inlineStr">
+        <is>
+          <t>RULE-COAST-TO-COAST</t>
+        </is>
+      </c>
+      <c r="B13" s="3" t="inlineStr">
+        <is>
+          <t>Coast-to-coast multi-DC optimization</t>
+        </is>
+      </c>
+      <c r="C13" s="3" t="inlineStr">
+        <is>
+          <t>DC-CHI-01</t>
+        </is>
+      </c>
+      <c r="D13" s="3" t="inlineStr">
+        <is>
+          <t>DC-LA-05,DC-DET-02</t>
+        </is>
+      </c>
+      <c r="E13" s="3" t="inlineStr"/>
+      <c r="F13" s="3" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="G13" s="3" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="H13" s="3" t="n">
+        <v>10</v>
+      </c>
+      <c r="I13" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="J13" s="3" t="n">
+        <v>7</v>
+      </c>
+      <c r="K13" s="3" t="inlineStr">
+        <is>
+          <t>GOLD</t>
+        </is>
+      </c>
+      <c r="L13" s="3" t="inlineStr">
+        <is>
+          <t>Project sites reachable from Chicago (preferred), Los Angeles, or Detroit. Optimization stage evaluates all three, splits allowed. Winner is chosen by lowest freight cost among feasible plans meeting the 7-day SLA.</t>
         </is>
       </c>
     </row>

</xml_diff>